<commit_message>
feat: bind editable Excel charts to dataset sheets
</commit_message>
<xml_diff>
--- a/src/test/resources/fixtures/templates/report-template.xlsx
+++ b/src/test/resources/fixtures/templates/report-template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>研发效能报告模板</t>
   </si>
@@ -49,6 +49,27 @@
   </si>
   <si>
     <t>附件：approval-detail.xlsx</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>uncertain</t>
+  </si>
+  <si>
+    <t>certain</t>
+  </si>
+  <si>
+    <t>baseline</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
   </si>
 </sst>
 </file>
@@ -105,6 +126,321 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr anchor="t" rtlCol="false"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l">
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="zh-CN"/>
+              <a:t>中心事件数</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1100"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="false"/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>报表首页!$G$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>不定责事件</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dLbls>
+            <c:showLegendKey val="false"/>
+            <c:showVal val="true"/>
+            <c:showCatName val="false"/>
+            <c:showSerName val="false"/>
+            <c:showPercent val="false"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'报表首页'!$F$16:$F$18</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2026年1月</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2026年2月</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2026年3月</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'报表首页'!$G$16:$G$18</c:f>
+              <c:numCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>报表首页!$H$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>定责事件</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dLbls>
+            <c:showLegendKey val="false"/>
+            <c:showVal val="true"/>
+            <c:showCatName val="false"/>
+            <c:showSerName val="false"/>
+            <c:showPercent val="false"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'报表首页'!$F$16:$F$18</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2026年1月</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2026年2月</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2026年3月</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'报表首页'!$H$16:$H$18</c:f>
+              <c:numCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:overlap val="100"/>
+        <c:axId val="0"/>
+        <c:axId val="1"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>报表首页!$I$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>中心基准值</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:showLegendKey val="false"/>
+            <c:showVal val="true"/>
+            <c:showCatName val="false"/>
+            <c:showSerName val="false"/>
+            <c:showPercent val="false"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'报表首页'!$F$16:$F$18</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2026年1月</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2026年2月</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2026年3月</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'报表首页'!$I$16:$I$18</c:f>
+              <c:numCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>12.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="2"/>
+        <c:axId val="3"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="0"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="false"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="false"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="false"/>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="0"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="true"/>
+        <c:axPos val="t"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="3"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="false"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="3"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="false"/>
+        <c:axPos val="r"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="false"/>
+    </c:legend>
+    <c:plotVisOnly val="false"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="0" name="Diagramm0" descr="REPORT_CHART:centerEventChart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="5334000" cy="3810000"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" ref="A3:B5" displayName="tbl_center_monthly" name="tbl_center_monthly">
   <tableColumns count="2">
@@ -125,8 +461,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -134,8 +470,65 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15">
+      <c r="F15" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H15" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I15" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="F16" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G16" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="H16" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="I16" t="n" s="0">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="F17" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="G17" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="H17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="I17" t="n" s="0">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="F18" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="G18" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H18" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="I18" t="n" s="0">
+        <v>2.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -144,8 +537,8 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="18.0" customWidth="true"/>
-    <col min="2" max="2" width="14.0" customWidth="true"/>
+    <col min="1" max="1" customWidth="true" width="18.0"/>
+    <col min="2" max="2" customWidth="true" width="14.0"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>